<commit_message>
Add .gitignore to datasets and updated documentation
</commit_message>
<xml_diff>
--- a/docs/datasets/dataset_inventory.xlsx
+++ b/docs/datasets/dataset_inventory.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\varun\Harbinger\data\datasets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\varun\Harbinger\docs\datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7DFB5FC-8C54-41FA-BE4F-8DBF5B204E6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ED9429D-0C2F-44B1-A850-CAB834325766}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30612" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="42144" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Dataset</t>
   </si>
@@ -61,13 +61,90 @@
   </si>
   <si>
     <t>Google Cluster Trace (optional)</t>
+  </si>
+  <si>
+    <t>Microsoft Research</t>
+  </si>
+  <si>
+    <t>DNN Training / GPU Cluster Traces</t>
+  </si>
+  <si>
+    <t>Yes (Local)</t>
+  </si>
+  <si>
+    <t>0.98 GB (Zip) / 6.6 GB (Raw)</t>
+  </si>
+  <si>
+    <t>JSON &amp; CSV</t>
+  </si>
+  <si>
+    <r>
+      <t>Yes (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Pass</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Killed</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Failed</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <t>2-month trace containing over 117,000 job logs.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -82,6 +159,11 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="2">
@@ -116,7 +198,30 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -127,6 +232,23 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2B2CCFE5-0679-4E96-9469-513E3C5A4369}" name="Table1" displayName="Table1" ref="B2:I6" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="B2:I6" xr:uid="{2B2CCFE5-0679-4E96-9469-513E3C5A4369}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{A86BA723-8D03-4BBA-B101-C5B162A14A6B}" name="Dataset" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{F06B1663-A506-4631-AA6D-FE1606DF5E91}" name="Source"/>
+    <tableColumn id="3" xr3:uid="{EAB31DBE-301D-4F78-8FD9-45B61C33E907}" name="Domain"/>
+    <tableColumn id="4" xr3:uid="{3AAE4FA3-1393-4902-97A9-1646CD9C3773}" name="Downloaded"/>
+    <tableColumn id="5" xr3:uid="{7DCA69BA-93F2-4913-970E-DBDCF95B7018}" name="File Size"/>
+    <tableColumn id="6" xr3:uid="{A2DC17E2-DC0B-4570-86D4-1BC1D3E2560C}" name="Format"/>
+    <tableColumn id="7" xr3:uid="{7D6D91D5-C3EA-40E4-8204-E0A9568FCC19}" name="Failure Labels"/>
+    <tableColumn id="8" xr3:uid="{EDFC1E18-85F6-4C95-AD97-3E1F6B46E6CC}" name="Notes"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -393,9 +515,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:I6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.85546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="2" spans="2:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:9">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -421,27 +553,51 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="2:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:9" ht="30">
       <c r="B3" s="2" t="s">
         <v>8</v>
       </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I3" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="4" spans="2:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:9" ht="45">
       <c r="B4" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:9">
       <c r="B5" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="2:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:9" ht="60">
       <c r="B6" s="2" t="s">
         <v>11</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>